<commit_message>
Update latest evolutions result
</commit_message>
<xml_diff>
--- a/latest/evolutions_raw_latest.xlsx
+++ b/latest/evolutions_raw_latest.xlsx
@@ -1135,7 +1135,7 @@
       </c>
       <c r="DA2" t="inlineStr">
         <is>
-          <t>Intro to Repeatable Evolutions 2 Discover Repeatable Evolutions, allowing you to run multiple players through the same upgrade path! Ioannidis 76 ST PAC 77 SHO 75 PAS 62 DRI 77 DEF 35 PHY 77 R 3 ★ 4 ST 76.3 Ioannidis 77 ST PAC 77 SHO 77 PAS 65 DRI 78 DEF 35 PHY 77 R 3 ★ 4 ST 77.1 REQUIREMENTS Overall Max. 79 Position ST Pace Max. 81 UPGRADES +1 OVR 80 +4 Long Shots 77 +3 Vision 79 +3 Short Pass 78 +4 Reactions 80 +3 Shot Power 78 +3 Volleys 78 +4 Fk Accuracy 80 +4 Long Pass 77 +4 Dribbling 80 in 1 year in 1 year 89% 11%</t>
+          <t>Intro to Repeatable Evolutions 2 Discover Repeatable Evolutions, allowing you to run multiple players through the same upgrade path! Ioannidis 76 ST PAC 77 SHO 75 PAS 62 DRI 77 DEF 35 PHY 77 R 3 ★ 4 ST 76.3 Ioannidis 77 ST PAC 77 SHO 77 PAS 65 DRI 78 DEF 35 PHY 77 R 3 ★ 4 ST 77.1 REQUIREMENTS Overall Max. 79 Position ST Pace Max. 81 UPGRADES +1 OVR 80 +4 Long Shots 77 +3 Vision 79 +3 Short Pass 78 +4 Reactions 80 +3 Shot Power 78 +3 Volleys 78 +4 Fk Accuracy 80 +4 Long Pass 77 +4 Dribbling 80 in 1 year in 1 year 88% 12%</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="DA3" t="inlineStr">
         <is>
-          <t>Intro to Evolutions Welcome to Evolutions in FC 27! Upgrade a player of your choice and unlock their first attribute boost. Trimmel 75 RB PAC 61 SHO 65 PAS 74 DRI 68 DEF 74 PHY 79 RM R 3 ★ 3 RB 63.4 Trimmel 79 RB PAC 80 SHO 65 PAS 77 DRI 79 DEF 76 PHY 81 RM R 3 ★ 3 RB 76.7 REQUIREMENTS Max Pos. 2 Overall Max. 75 Position RB Excluded Position CB Max PS 7 Pace Max. 80 UPGRADES +34 OVR 79 +40 Sprint Speed 80 +40 Short Pass 76 +40 Balance 77 +40 Interceptions 76 +40 Sliding Tackle 75 +40 Vision 75 +40 Curve 80 +40 Ball Control 80 +40 Defensive Awareness 77 +40 Stamina 80 +40 Acceleration 80 +40 Crossing 78 +40 Agility 78 +40 Dribbling 80 +40 Standing Tackle 78 RB Wingback + 3 in 1 year in 1 year 92% 8%</t>
+          <t>Intro to Evolutions Welcome to Evolutions in FC 27! Upgrade a player of your choice and unlock their first attribute boost. Trimmel 75 RB PAC 61 SHO 65 PAS 74 DRI 68 DEF 74 PHY 79 RM R 3 ★ 3 RB 63.4 Trimmel 79 RB PAC 80 SHO 65 PAS 77 DRI 79 DEF 76 PHY 81 RM R 3 ★ 3 RB 76.7 REQUIREMENTS Max Pos. 2 Overall Max. 75 Position RB Excluded Position CB Max PS 7 Pace Max. 80 UPGRADES +34 OVR 79 +40 Sprint Speed 80 +40 Short Pass 76 +40 Balance 77 +40 Interceptions 76 +40 Sliding Tackle 75 +40 Vision 75 +40 Curve 80 +40 Ball Control 80 +40 Defensive Awareness 77 +40 Stamina 80 +40 Acceleration 80 +40 Crossing 78 +40 Agility 78 +40 Dribbling 80 +40 Standing Tackle 78 RB Wingback + 3 in 1 year in 1 year 93% 8%</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="DA4" t="inlineStr">
         <is>
-          <t>Intro to Training Camp EVOs Send your players to training camp! Collect their attribute upgrades when the training session concludes. Antônia Silva 80 RB PAC 81 SHO 50 PAS 71 DRI 79 DEF 79 PHY 79 RM R 4 ★ 3 RB 75.5 Antônia Silva 80 RB PAC 81 SHO 50 PAS 71 DRI 79 DEF 79 PHY 79 RM R 4 ★ 3 RB 78.4 REQUIREMENTS Overall Max. 80 Position RB UPGRADES RB Fullback + TRAINING TIME 1 hours in 1 year in 1 year 91% 9%</t>
+          <t>Intro to Training Camp EVOs Send your players to training camp! Collect their attribute upgrades when the training session concludes. REQUIREMENTS Overall Max. 80 Position RB UPGRADES RB Fullback + TRAINING TIME 1 hours in 1 year in 1 year 91% 9%</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       <c r="CV6" t="inlineStr"/>
       <c r="CW6" t="inlineStr">
         <is>
-          <t>! OVERVIEW ELIGIBLE PLAYERS EVOLVED PLAYERS TRENDING EVOLVED PLAYERS Community Verdict Worth Doing 88% of GG users upvoted this Evolution. Vote Now! 88% 12% Completion Difficulty Easy Number of Games 1 Recommended Position RW Number of Wins 0 Is Your Player Eligible? Want to check eligibility for your already evolved players? Sync them now on GG Club Trending Evolved Players View All Evolution Upgrades 4 Level 1 Fofana 80 CM PAC 75 SHO 69 PAS 76 DRI 79 DEF 78 PHY 74 CAM R 3 ★ 3 Fofana 80 CM PAC 75 SHO 69 PAS 76 DRI 79 DEF 78 PHY 74 CAM R 3 ★ 3 UPGRADE PATHS Pick one Option A 76.8 GGR 4 Option B Best GG Rating 77.0 GGR 4</t>
+          <t>! OVERVIEW ELIGIBLE PLAYERS EVOLVED PLAYERS TRENDING EVOLVED PLAYERS Community Verdict Worth Doing 89% of GG users upvoted this Evolution. Vote Now! 89% 11% Completion Difficulty Easy Number of Games 1 Recommended Position RW Number of Wins 0 Is Your Player Eligible? Want to check eligibility for your already evolved players? Sync them now on GG Club Trending Evolved Players View All Evolution Upgrades 4 Level 1 Fofana 80 CM PAC 75 SHO 69 PAS 76 DRI 79 DEF 78 PHY 74 CAM R 3 ★ 3 Fofana 80 CM PAC 75 SHO 69 PAS 76 DRI 79 DEF 78 PHY 74 CAM R 3 ★ 3 UPGRADE PATHS Pick one Option A 77.0 GGR 4 Option B Best GG Rating 77.2 GGR 4</t>
         </is>
       </c>
       <c r="CX6" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="DA6" t="inlineStr">
         <is>
-          <t>Intro to Pathway Evolutions Explore Pathway Evolutions, a new type of Evolution that allows you to choose how your player develops and upgrades! Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 82.1 Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 83.2 REQUIREMENTS Overall Max. 80 Max PS 3 UPGRADES 4 in 1 year in 1 year 88% 12%</t>
+          <t>Intro to Pathway Evolutions Explore Pathway Evolutions, a new type of Evolution that allows you to choose how your player develops and upgrades! Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 82.1 Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 83.2 REQUIREMENTS Overall Max. 80 Max PS 3 UPGRADES 4 in 1 year in 1 year 89% 11%</t>
         </is>
       </c>
     </row>
@@ -2053,12 +2053,12 @@
       </c>
       <c r="CZ7" t="inlineStr">
         <is>
-          <t>Pinged Pass NEW</t>
+          <t>Pinged Pass</t>
         </is>
       </c>
       <c r="DA7" t="inlineStr">
         <is>
-          <t>Pinged Pass NEW Unlocked by completing the Pep's Domination task in the Ones We Watched World Class Challenge objective Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 78.2 Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 79.2 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Pinged Pass Unlocked by completing the Pep's Domination task in the Ones We Watched World Class Challenge objective Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 78.2 Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 79.2 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
         </is>
       </c>
     </row>
@@ -2216,12 +2216,12 @@
       </c>
       <c r="CZ8" t="inlineStr">
         <is>
-          <t>Believe NEW</t>
+          <t>Believe</t>
         </is>
       </c>
       <c r="DA8" t="inlineStr">
         <is>
-          <t>Believe NEW Unlocked by completing the Ted Lasso's Masterclass objective Olaru 73 CM PAC 84 SHO 75 PAS 73 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 81.7 Olaru 74 CM PAC 84 SHO 75 PAS 74 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 82.2 REQUIREMENTS Overall Max. 82 Position ST UPGRADES +1 OVR 83 +4 Short Pass 83 +3 Composure 84 in 1 year in 1 year 25% 75%</t>
+          <t>Believe Unlocked by completing the Ted Lasso's Masterclass objective Olaru 73 CM PAC 84 SHO 75 PAS 73 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 81.7 Olaru 74 CM PAC 84 SHO 75 PAS 74 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 82.2 REQUIREMENTS Overall Max. 82 Position ST UPGRADES +1 OVR 83 +4 Short Pass 83 +3 Composure 84 in 1 year in 1 year 27% 73%</t>
         </is>
       </c>
     </row>
@@ -2375,12 +2375,12 @@
       </c>
       <c r="CZ9" t="inlineStr">
         <is>
-          <t>Shooting Practice [SP+ 28] NEW</t>
+          <t>Shooting Practice [SP+ 28]</t>
         </is>
       </c>
       <c r="DA9" t="inlineStr">
         <is>
-          <t>Shooting Practice [SP+ 28] NEW Unlocked by reaching level 28 in the Premium Season Pass. Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 LM 79.5 Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 ST 81.3 REQUIREMENTS Overall Max. 81 Position LW, RW, ST Max PS 3 Max PS+ 0 UPGRADES 4 in 1 month in 1 month 83% 17%</t>
+          <t>Shooting Practice [SP+ 28] Unlocked by reaching level 28 in the Premium Season Pass. Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 LM 79.5 Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 ST 81.3 REQUIREMENTS Overall Max. 81 Position LW, RW, ST Max PS 3 Max PS+ 0 UPGRADES 4 in 1 month in 1 month 83% 17%</t>
         </is>
       </c>
     </row>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="CZ10" t="inlineStr">
         <is>
-          <t>Creative or Composed? [SP 27] NEW</t>
+          <t>Creative or Composed? [SP 27]</t>
         </is>
       </c>
       <c r="DA10" t="inlineStr">
         <is>
-          <t>Creative or Composed? [SP 27] NEW Unlocked by reaching level 27 in the Standard Season Pass. Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 78.2 Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 79.6 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Creative or Composed? [SP 27] Unlocked by reaching level 27 in the Standard Season Pass. Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 78.2 Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 79.6 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
         </is>
       </c>
     </row>
@@ -2785,12 +2785,12 @@
       </c>
       <c r="CZ11" t="inlineStr">
         <is>
-          <t>Winger Glow Up [SP+ 26] NEW</t>
+          <t>Winger Glow Up [SP+ 26]</t>
         </is>
       </c>
       <c r="DA11" t="inlineStr">
         <is>
-          <t>Winger Glow Up [SP+ 26] NEW Unlocked by reaching level 26 in the Premium Season Pass. Di Francesco 72 LM PAC 73 SHO 69 PAS 71 DRI 74 DEF 51 PHY 60 LW R 4 ★ 4 LW 70.5 Di Francesco 82 LM PAC 85 SHO 77 PAS 78 DRI 84 DEF 51 PHY 62 LW R 4 ★ 4 LM 81.5 REQUIREMENTS Max Pos. 3 Overall Max. 81 Position LW Excluded Position LB, ST Max PS 7 Max PS+ 0 Pace Max. 85 UPGRADES +10 OVR 83 +1 SM 3 +10 Positioning 80 +10 Volleys 74 +10 Fk Accuracy 73 +15 Agility 86 +15 Dribbling 84 +10 Finishing 78 +10 Penalties 74 +10 Short Pass 76 +15 Balance 85 +15 Composure 80 +15 Acceleration 85 +10 Shot Power 77 +10 Vision 81 +10 Long Pass 80 +15 Reactions 78 +10 Stamina 72 +15 Sprint Speed 85 +10 Long Shots 80 +10 Crossing 82 +10 Curve 78 +15 Ball Control 85 3 in 1 month in 1 month 83% 17%</t>
+          <t>Winger Glow Up [SP+ 26] Unlocked by reaching level 26 in the Premium Season Pass. Di Francesco 72 LM PAC 73 SHO 69 PAS 71 DRI 74 DEF 51 PHY 60 LW R 4 ★ 4 LW 70.5 Di Francesco 82 LM PAC 85 SHO 77 PAS 78 DRI 84 DEF 51 PHY 62 LW R 4 ★ 4 LM 81.5 REQUIREMENTS Max Pos. 3 Overall Max. 81 Position LW Excluded Position LB, ST Max PS 7 Max PS+ 0 Pace Max. 85 UPGRADES +10 OVR 83 +1 SM 3 +10 Positioning 80 +10 Volleys 74 +10 Fk Accuracy 73 +15 Agility 86 +15 Dribbling 84 +10 Finishing 78 +10 Penalties 74 +10 Short Pass 76 +15 Balance 85 +15 Composure 80 +15 Acceleration 85 +10 Shot Power 77 +10 Vision 81 +10 Long Pass 80 +15 Reactions 78 +10 Stamina 72 +15 Sprint Speed 85 +10 Long Shots 80 +10 Crossing 82 +10 Curve 78 +15 Ball Control 85 3 in 1 month in 1 month 92% 8%</t>
         </is>
       </c>
     </row>
@@ -2936,12 +2936,12 @@
       </c>
       <c r="CZ12" t="inlineStr">
         <is>
-          <t>Tactical Ascent [SP+ 14] NEW</t>
+          <t>Tactical Ascent [SP+ 14]</t>
         </is>
       </c>
       <c r="DA12" t="inlineStr">
         <is>
-          <t>Tactical Ascent [SP+ 14] NEW Unlocked by reaching level 14 in the Premium Season Pass. Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 77.3 Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 80.0 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 80% 20%</t>
+          <t>Tactical Ascent [SP+ 14] Unlocked by reaching level 14 in the Premium Season Pass. Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 77.3 Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 80.0 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 90% 10%</t>
         </is>
       </c>
     </row>
@@ -3087,12 +3087,12 @@
       </c>
       <c r="CZ13" t="inlineStr">
         <is>
-          <t>Relentless [SP 11] NEW</t>
+          <t>Relentless [SP 11]</t>
         </is>
       </c>
       <c r="DA13" t="inlineStr">
         <is>
-          <t>Relentless [SP 11] NEW Unlocked by reaching level 11 in the Standard Season Pass. Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.3 Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.9 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Relentless [SP 11] Unlocked by reaching level 11 in the Standard Season Pass. Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.3 Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.9 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 33% 67%</t>
         </is>
       </c>
     </row>
@@ -3338,12 +3338,12 @@
       </c>
       <c r="CZ14" t="inlineStr">
         <is>
-          <t>Striker Glow Up [SP 7] NEW</t>
+          <t>Striker Glow Up [SP 7]</t>
         </is>
       </c>
       <c r="DA14" t="inlineStr">
         <is>
-          <t>Striker Glow Up [SP 7] NEW Unlocked by reaching level 7 in the Standard Season Pass. Mugoša 74 ST PAC 71 SHO 75 PAS 56 DRI 67 DEF 26 PHY 81 R 3 ★ 4 ST 69.8 Mugoša 80 ST PAC 78 SHO 81 PAS 62 DRI 75 DEF 26 PHY 81 R 3 ★ 4 ST 77.9 REQUIREMENTS Max Pos. 3 Overall Max. 79 Position ST Excluded Position CAM, CM Max PS 7 Pace Max. 84 UPGRADES +10 OVR 80 +15 Positioning 82 +15 Volleys 78 +8 Long Pass 62 +10 Reactions 76 +10 Jumping 78 +15 Finishing 83 +10 Penalties 75 +15 Curve 77 +10 Ball Control 76 +10 Stamina 67 +10 Acceleration 80 +15 Shot Power 82 +8 Vision 70 +15 Agility 78 +10 Dribbling 76 +10 Sprint Speed 78 +15 Long Shots 78 +8 Short Pass 72 +15 Balance 77 +8 Composure 80 3 in 1 month in 1 month 100% 0%</t>
+          <t>Striker Glow Up [SP 7] Unlocked by reaching level 7 in the Standard Season Pass. Mugoša 74 ST PAC 71 SHO 75 PAS 56 DRI 67 DEF 26 PHY 81 R 3 ★ 4 ST 69.8 Mugoša 80 ST PAC 78 SHO 81 PAS 62 DRI 75 DEF 26 PHY 81 R 3 ★ 4 ST 77.9 REQUIREMENTS Max Pos. 3 Overall Max. 79 Position ST Excluded Position CAM, CM Max PS 7 Pace Max. 84 UPGRADES +10 OVR 80 +15 Positioning 82 +15 Volleys 78 +8 Long Pass 62 +10 Reactions 76 +10 Jumping 78 +15 Finishing 83 +10 Penalties 75 +15 Curve 77 +10 Ball Control 76 +10 Stamina 67 +10 Acceleration 80 +15 Shot Power 82 +8 Vision 70 +15 Agility 78 +10 Dribbling 76 +10 Sprint Speed 78 +15 Long Shots 78 +8 Short Pass 72 +15 Balance 77 +8 Composure 80 3 in 1 month in 1 month 91% 9%</t>
         </is>
       </c>
     </row>
@@ -3505,12 +3505,12 @@
       </c>
       <c r="CZ15" t="inlineStr">
         <is>
-          <t>Midfield Polish [SP+ 1] NEW</t>
+          <t>Midfield Polish [SP+ 1]</t>
         </is>
       </c>
       <c r="DA15" t="inlineStr">
         <is>
-          <t>Midfield Polish [SP+ 1] NEW Unlocked by reaching level 1 in the Premium Season Pass. Moreno 78 CDM PAC 81 SHO 68 PAS 73 DRI 76 DEF 76 PHY 77 CM R 4 ★ 3 CDM 78.9 Moreno 79 CDM PAC 81 SHO 68 PAS 74 DRI 76 DEF 77 PHY 77 CM R 4 ★ 3 CDM 79.4 REQUIREMENTS Overall Max. 79 Position CM, CDM Excluded Position CAM UPGRADES +1 OVR 80 +1 PAS 79 +1 DEF 79 in 1 month in 1 month 43% 57%</t>
+          <t>Midfield Polish [SP+ 1] Unlocked by reaching level 1 in the Premium Season Pass. Moreno 78 CDM PAC 81 SHO 68 PAS 73 DRI 76 DEF 76 PHY 77 CM R 4 ★ 3 CDM 78.9 Moreno 79 CDM PAC 81 SHO 68 PAS 74 DRI 76 DEF 77 PHY 77 CM R 4 ★ 3 CDM 79.4 REQUIREMENTS Overall Max. 79 Position CM, CDM Excluded Position CAM UPGRADES +1 OVR 80 +1 PAS 79 +1 DEF 79 in 1 month in 1 month 27% 73%</t>
         </is>
       </c>
     </row>
@@ -10097,7 +10097,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Intro to Repeatable Evolutions 2 Discover Repeatable Evolutions, allowing you to run multiple players through the same upgrade path! Ioannidis 76 ST PAC 77 SHO 75 PAS 62 DRI 77 DEF 35 PHY 77 R 3 ★ 4 ST 76.3 Ioannidis 77 ST PAC 77 SHO 77 PAS 65 DRI 78 DEF 35 PHY 77 R 3 ★ 4 ST 77.1 REQUIREMENTS Overall Max. 79 Position ST Pace Max. 81 UPGRADES +1 OVR 80 +4 Long Shots 77 +3 Vision 79 +3 Short Pass 78 +4 Reactions 80 +3 Shot Power 78 +3 Volleys 78 +4 Fk Accuracy 80 +4 Long Pass 77 +4 Dribbling 80 in 1 year in 1 year 89% 11%</t>
+          <t>Intro to Repeatable Evolutions 2 Discover Repeatable Evolutions, allowing you to run multiple players through the same upgrade path! Ioannidis 76 ST PAC 77 SHO 75 PAS 62 DRI 77 DEF 35 PHY 77 R 3 ★ 4 ST 76.3 Ioannidis 77 ST PAC 77 SHO 77 PAS 65 DRI 78 DEF 35 PHY 77 R 3 ★ 4 ST 77.1 REQUIREMENTS Overall Max. 79 Position ST Pace Max. 81 UPGRADES +1 OVR 80 +4 Long Shots 77 +3 Vision 79 +3 Short Pass 78 +4 Reactions 80 +3 Shot Power 78 +3 Volleys 78 +4 Fk Accuracy 80 +4 Long Pass 77 +4 Dribbling 80 in 1 year in 1 year 88% 12%</t>
         </is>
       </c>
     </row>
@@ -10124,7 +10124,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Intro to Evolutions Welcome to Evolutions in FC 27! Upgrade a player of your choice and unlock their first attribute boost. Trimmel 75 RB PAC 61 SHO 65 PAS 74 DRI 68 DEF 74 PHY 79 RM R 3 ★ 3 RB 63.4 Trimmel 79 RB PAC 80 SHO 65 PAS 77 DRI 79 DEF 76 PHY 81 RM R 3 ★ 3 RB 76.7 REQUIREMENTS Max Pos. 2 Overall Max. 75 Position RB Excluded Position CB Max PS 7 Pace Max. 80 UPGRADES +34 OVR 79 +40 Sprint Speed 80 +40 Short Pass 76 +40 Balance 77 +40 Interceptions 76 +40 Sliding Tackle 75 +40 Vision 75 +40 Curve 80 +40 Ball Control 80 +40 Defensive Awareness 77 +40 Stamina 80 +40 Acceleration 80 +40 Crossing 78 +40 Agility 78 +40 Dribbling 80 +40 Standing Tackle 78 RB Wingback + 3 in 1 year in 1 year 92% 8%</t>
+          <t>Intro to Evolutions Welcome to Evolutions in FC 27! Upgrade a player of your choice and unlock their first attribute boost. Trimmel 75 RB PAC 61 SHO 65 PAS 74 DRI 68 DEF 74 PHY 79 RM R 3 ★ 3 RB 63.4 Trimmel 79 RB PAC 80 SHO 65 PAS 77 DRI 79 DEF 76 PHY 81 RM R 3 ★ 3 RB 76.7 REQUIREMENTS Max Pos. 2 Overall Max. 75 Position RB Excluded Position CB Max PS 7 Pace Max. 80 UPGRADES +34 OVR 79 +40 Sprint Speed 80 +40 Short Pass 76 +40 Balance 77 +40 Interceptions 76 +40 Sliding Tackle 75 +40 Vision 75 +40 Curve 80 +40 Ball Control 80 +40 Defensive Awareness 77 +40 Stamina 80 +40 Acceleration 80 +40 Crossing 78 +40 Agility 78 +40 Dribbling 80 +40 Standing Tackle 78 RB Wingback + 3 in 1 year in 1 year 93% 8%</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10151,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Intro to Training Camp EVOs Send your players to training camp! Collect their attribute upgrades when the training session concludes. Antônia Silva 80 RB PAC 81 SHO 50 PAS 71 DRI 79 DEF 79 PHY 79 RM R 4 ★ 3 RB 75.5 Antônia Silva 80 RB PAC 81 SHO 50 PAS 71 DRI 79 DEF 79 PHY 79 RM R 4 ★ 3 RB 78.4 REQUIREMENTS Overall Max. 80 Position RB UPGRADES RB Fullback + TRAINING TIME 1 hours in 1 year in 1 year 91% 9%</t>
+          <t>Intro to Training Camp EVOs Send your players to training camp! Collect their attribute upgrades when the training session concludes. REQUIREMENTS Overall Max. 80 Position RB UPGRADES RB Fullback + TRAINING TIME 1 hours in 1 year in 1 year 91% 9%</t>
         </is>
       </c>
     </row>
@@ -10205,7 +10205,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Intro to Pathway Evolutions Explore Pathway Evolutions, a new type of Evolution that allows you to choose how your player develops and upgrades! Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 82.1 Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 83.2 REQUIREMENTS Overall Max. 80 Max PS 3 UPGRADES 4 in 1 year in 1 year 88% 12%</t>
+          <t>Intro to Pathway Evolutions Explore Pathway Evolutions, a new type of Evolution that allows you to choose how your player develops and upgrades! Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 82.1 Chiesa 80 RM PAC 87 SHO 79 PAS 75 DRI 83 DEF 44 PHY 68 RW ST R 4 ★ 4 RM 83.2 REQUIREMENTS Overall Max. 80 Max PS 3 UPGRADES 4 in 1 year in 1 year 89% 11%</t>
         </is>
       </c>
     </row>
@@ -10227,12 +10227,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Pinged Pass NEW</t>
+          <t>Pinged Pass</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Pinged Pass NEW Unlocked by completing the Pep's Domination task in the Ones We Watched World Class Challenge objective Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 78.2 Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 79.2 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Pinged Pass Unlocked by completing the Pep's Domination task in the Ones We Watched World Class Challenge objective Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 78.2 Javi Guerra 77 CM PAC 74 SHO 73 PAS 75 DRI 76 DEF 74 PHY 75 CDM CAM R 3 ★ 4 CM 79.2 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
         </is>
       </c>
     </row>
@@ -10254,12 +10254,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Believe NEW</t>
+          <t>Believe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Believe NEW Unlocked by completing the Ted Lasso's Masterclass objective Olaru 73 CM PAC 84 SHO 75 PAS 73 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 81.7 Olaru 74 CM PAC 84 SHO 75 PAS 74 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 82.2 REQUIREMENTS Overall Max. 82 Position ST UPGRADES +1 OVR 83 +4 Short Pass 83 +3 Composure 84 in 1 year in 1 year 25% 75%</t>
+          <t>Believe Unlocked by completing the Ted Lasso's Masterclass objective Olaru 73 CM PAC 84 SHO 75 PAS 73 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 81.7 Olaru 74 CM PAC 84 SHO 75 PAS 74 DRI 75 DEF 66 PHY 77 CDM CAM ST R 3 ★ 5 CM 82.2 REQUIREMENTS Overall Max. 82 Position ST UPGRADES +1 OVR 83 +4 Short Pass 83 +3 Composure 84 in 1 year in 1 year 27% 73%</t>
         </is>
       </c>
     </row>
@@ -10281,12 +10281,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Shooting Practice [SP+ 28] NEW</t>
+          <t>Shooting Practice [SP+ 28]</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Shooting Practice [SP+ 28] NEW Unlocked by reaching level 28 in the Premium Season Pass. Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 LM 79.5 Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 ST 81.3 REQUIREMENTS Overall Max. 81 Position LW, RW, ST Max PS 3 Max PS+ 0 UPGRADES 4 in 1 month in 1 month 83% 17%</t>
+          <t>Shooting Practice [SP+ 28] Unlocked by reaching level 28 in the Premium Season Pass. Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 LM 79.5 Rahimi 78 ST PAC 87 SHO 78 PAS 71 DRI 79 DEF 38 PHY 68 RM LM RW LW R 4 ★ 4 ST 81.3 REQUIREMENTS Overall Max. 81 Position LW, RW, ST Max PS 3 Max PS+ 0 UPGRADES 4 in 1 month in 1 month 83% 17%</t>
         </is>
       </c>
     </row>
@@ -10308,12 +10308,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Creative or Composed? [SP 27] NEW</t>
+          <t>Creative or Composed? [SP 27]</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Creative or Composed? [SP 27] NEW Unlocked by reaching level 27 in the Standard Season Pass. Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 78.2 Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 79.6 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Creative or Composed? [SP 27] Unlocked by reaching level 27 in the Standard Season Pass. Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 78.2 Sow 76 CM PAC 76 SHO 73 PAS 73 DRI 75 DEF 74 PHY 78 CDM R 3 ★ 4 CM 79.6 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
         </is>
       </c>
     </row>
@@ -10335,12 +10335,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Winger Glow Up [SP+ 26] NEW</t>
+          <t>Winger Glow Up [SP+ 26]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Winger Glow Up [SP+ 26] NEW Unlocked by reaching level 26 in the Premium Season Pass. Di Francesco 72 LM PAC 73 SHO 69 PAS 71 DRI 74 DEF 51 PHY 60 LW R 4 ★ 4 LW 70.5 Di Francesco 82 LM PAC 85 SHO 77 PAS 78 DRI 84 DEF 51 PHY 62 LW R 4 ★ 4 LM 81.5 REQUIREMENTS Max Pos. 3 Overall Max. 81 Position LW Excluded Position LB, ST Max PS 7 Max PS+ 0 Pace Max. 85 UPGRADES +10 OVR 83 +1 SM 3 +10 Positioning 80 +10 Volleys 74 +10 Fk Accuracy 73 +15 Agility 86 +15 Dribbling 84 +10 Finishing 78 +10 Penalties 74 +10 Short Pass 76 +15 Balance 85 +15 Composure 80 +15 Acceleration 85 +10 Shot Power 77 +10 Vision 81 +10 Long Pass 80 +15 Reactions 78 +10 Stamina 72 +15 Sprint Speed 85 +10 Long Shots 80 +10 Crossing 82 +10 Curve 78 +15 Ball Control 85 3 in 1 month in 1 month 83% 17%</t>
+          <t>Winger Glow Up [SP+ 26] Unlocked by reaching level 26 in the Premium Season Pass. Di Francesco 72 LM PAC 73 SHO 69 PAS 71 DRI 74 DEF 51 PHY 60 LW R 4 ★ 4 LW 70.5 Di Francesco 82 LM PAC 85 SHO 77 PAS 78 DRI 84 DEF 51 PHY 62 LW R 4 ★ 4 LM 81.5 REQUIREMENTS Max Pos. 3 Overall Max. 81 Position LW Excluded Position LB, ST Max PS 7 Max PS+ 0 Pace Max. 85 UPGRADES +10 OVR 83 +1 SM 3 +10 Positioning 80 +10 Volleys 74 +10 Fk Accuracy 73 +15 Agility 86 +15 Dribbling 84 +10 Finishing 78 +10 Penalties 74 +10 Short Pass 76 +15 Balance 85 +15 Composure 80 +15 Acceleration 85 +10 Shot Power 77 +10 Vision 81 +10 Long Pass 80 +15 Reactions 78 +10 Stamina 72 +15 Sprint Speed 85 +10 Long Shots 80 +10 Crossing 82 +10 Curve 78 +15 Ball Control 85 3 in 1 month in 1 month 92% 8%</t>
         </is>
       </c>
     </row>
@@ -10362,12 +10362,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tactical Ascent [SP+ 14] NEW</t>
+          <t>Tactical Ascent [SP+ 14]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tactical Ascent [SP+ 14] NEW Unlocked by reaching level 14 in the Premium Season Pass. Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 77.3 Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 80.0 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 80% 20%</t>
+          <t>Tactical Ascent [SP+ 14] Unlocked by reaching level 14 in the Premium Season Pass. Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 77.3 Gorden 76 CB PAC 85 SHO 54 PAS 55 DRI 67 DEF 77 PHY 77 R 2 ★ 3 CB 80.0 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 90% 10%</t>
         </is>
       </c>
     </row>
@@ -10389,12 +10389,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Relentless [SP 11] NEW</t>
+          <t>Relentless [SP 11]</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Relentless [SP 11] NEW Unlocked by reaching level 11 in the Standard Season Pass. Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.3 Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.9 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 100% 0%</t>
+          <t>Relentless [SP 11] Unlocked by reaching level 11 in the Standard Season Pass. Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.3 Taylor 78 CM PAC 69 SHO 77 PAS 78 DRI 80 DEF 67 PHY 69 CDM L 3 ★ 5 CM 78.9 REQUIREMENTS Overall Max. 79 Max PS 2 UPGRADES 3 in 1 month in 1 month 33% 67%</t>
         </is>
       </c>
     </row>
@@ -10416,12 +10416,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Striker Glow Up [SP 7] NEW</t>
+          <t>Striker Glow Up [SP 7]</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Striker Glow Up [SP 7] NEW Unlocked by reaching level 7 in the Standard Season Pass. Mugoša 74 ST PAC 71 SHO 75 PAS 56 DRI 67 DEF 26 PHY 81 R 3 ★ 4 ST 69.8 Mugoša 80 ST PAC 78 SHO 81 PAS 62 DRI 75 DEF 26 PHY 81 R 3 ★ 4 ST 77.9 REQUIREMENTS Max Pos. 3 Overall Max. 79 Position ST Excluded Position CAM, CM Max PS 7 Pace Max. 84 UPGRADES +10 OVR 80 +15 Positioning 82 +15 Volleys 78 +8 Long Pass 62 +10 Reactions 76 +10 Jumping 78 +15 Finishing 83 +10 Penalties 75 +15 Curve 77 +10 Ball Control 76 +10 Stamina 67 +10 Acceleration 80 +15 Shot Power 82 +8 Vision 70 +15 Agility 78 +10 Dribbling 76 +10 Sprint Speed 78 +15 Long Shots 78 +8 Short Pass 72 +15 Balance 77 +8 Composure 80 3 in 1 month in 1 month 100% 0%</t>
+          <t>Striker Glow Up [SP 7] Unlocked by reaching level 7 in the Standard Season Pass. Mugoša 74 ST PAC 71 SHO 75 PAS 56 DRI 67 DEF 26 PHY 81 R 3 ★ 4 ST 69.8 Mugoša 80 ST PAC 78 SHO 81 PAS 62 DRI 75 DEF 26 PHY 81 R 3 ★ 4 ST 77.9 REQUIREMENTS Max Pos. 3 Overall Max. 79 Position ST Excluded Position CAM, CM Max PS 7 Pace Max. 84 UPGRADES +10 OVR 80 +15 Positioning 82 +15 Volleys 78 +8 Long Pass 62 +10 Reactions 76 +10 Jumping 78 +15 Finishing 83 +10 Penalties 75 +15 Curve 77 +10 Ball Control 76 +10 Stamina 67 +10 Acceleration 80 +15 Shot Power 82 +8 Vision 70 +15 Agility 78 +10 Dribbling 76 +10 Sprint Speed 78 +15 Long Shots 78 +8 Short Pass 72 +15 Balance 77 +8 Composure 80 3 in 1 month in 1 month 91% 9%</t>
         </is>
       </c>
     </row>
@@ -10443,12 +10443,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Midfield Polish [SP+ 1] NEW</t>
+          <t>Midfield Polish [SP+ 1]</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Midfield Polish [SP+ 1] NEW Unlocked by reaching level 1 in the Premium Season Pass. Moreno 78 CDM PAC 81 SHO 68 PAS 73 DRI 76 DEF 76 PHY 77 CM R 4 ★ 3 CDM 78.9 Moreno 79 CDM PAC 81 SHO 68 PAS 74 DRI 76 DEF 77 PHY 77 CM R 4 ★ 3 CDM 79.4 REQUIREMENTS Overall Max. 79 Position CM, CDM Excluded Position CAM UPGRADES +1 OVR 80 +1 PAS 79 +1 DEF 79 in 1 month in 1 month 43% 57%</t>
+          <t>Midfield Polish [SP+ 1] Unlocked by reaching level 1 in the Premium Season Pass. Moreno 78 CDM PAC 81 SHO 68 PAS 73 DRI 76 DEF 76 PHY 77 CM R 4 ★ 3 CDM 78.9 Moreno 79 CDM PAC 81 SHO 68 PAS 74 DRI 76 DEF 77 PHY 77 CM R 4 ★ 3 CDM 79.4 REQUIREMENTS Overall Max. 79 Position CM, CDM Excluded Position CAM UPGRADES +1 OVR 80 +1 PAS 79 +1 DEF 79 in 1 month in 1 month 27% 73%</t>
         </is>
       </c>
     </row>
@@ -10519,7 +10519,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-16T20:06:04</t>
+          <t>2026-09-17T20:18:50</t>
         </is>
       </c>
     </row>

</xml_diff>